<commit_message>
feat: TC-BILL-09/10 + TC-DASH-05 (50 cases, Newman 25/25)
</commit_message>
<xml_diff>
--- a/reports/KosManager-QA-Report.xlsx
+++ b/reports/KosManager-QA-Report.xlsx
@@ -494,7 +494,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>47/47 Pass</t>
+          <t>50/50 Pass</t>
         </is>
       </c>
     </row>
@@ -512,7 +512,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F48"/>
+  <dimension ref="A1:F51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2018,6 +2018,100 @@
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>TC-BILL-09</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>bills</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Struk PDF valid + milik sendiri</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>GET /api/bills/4/receipt.pdf token owner</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>200 application/pdf, magic bytes %PDF</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>TC-BILL-10</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>bills</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Struk tagihan orang lain 403</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>GET /api/bills/5/receipt.pdf token sinta</t>
+        </is>
+      </c>
+      <c r="E50" t="n">
+        <v>403</v>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>TC-DASH-05</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>dashboard</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Tren kas 6 bulan konsisten</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>GET /api/dashboard/trend, bandingkan vs dashboard</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>6 points, kas periode berjalan cocok</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -2102,7 +2196,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="C4" t="n">
         <v>0</v>
@@ -2215,7 +2309,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>22/22</t>
+          <t>25/25</t>
         </is>
       </c>
     </row>
@@ -2239,7 +2333,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>47/47</t>
+          <t>50/50</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: TC-NTF-06..09 polling (54 cases)
</commit_message>
<xml_diff>
--- a/reports/KosManager-QA-Report.xlsx
+++ b/reports/KosManager-QA-Report.xlsx
@@ -494,7 +494,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>50/50 Pass</t>
+          <t>54/54 Pass</t>
         </is>
       </c>
     </row>
@@ -512,7 +512,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F51"/>
+  <dimension ref="A1:F55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2112,6 +2112,134 @@
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>TC-NTF-06</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>notify</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Polling /start tautkan chat_id</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>fake updates /start sinta@kos.local, tunggu sweep</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>tenant.TelegramChatId terisi, offset maju</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>TC-NTF-07</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>notify</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Polling SUDAH buat pending payment</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>fake updates SUDAH setelah taut</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>1 payment pending untuk tagihan unpaid terbaru</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>TC-NTF-08</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>notify</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Redelivery idempoten</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>reset offset, sweep ulang</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>payment tetap 1, tanpa duplikat</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>TC-NTF-09</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>notify</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Email tak dikenal dibalas instruksi</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>fake /start asing@example.com</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>tanpa perubahan DB</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -2196,7 +2324,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="C4" t="n">
         <v>0</v>
@@ -2333,7 +2461,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>50/50</t>
+          <t>54/54</t>
         </is>
       </c>
     </row>

</xml_diff>